<commit_message>
SGG: Anadir agente bibliografico y proteger citas/vinetas no respaldadas
Engancha tarea_validacion_pdf al modo PDF de abstract (antes era codigo
muerto), refuerza los mismos chequeos de fidelidad ya usados en abstract
dentro del pipeline de introduccion, y anade marcar_citas_sin_respaldo()
en bib_writer.py: compara en codigo cada cita "Apellido (Año)" contra el
.bib real y marca con [VERIFICAR] las que no tengan paper detras, en vez
de depender de que el LLM se acuerde de no inventarlas.
</commit_message>
<xml_diff>
--- a/abstracts/comparacion_abstracts.xlsx
+++ b/abstracts/comparacion_abstracts.xlsx
@@ -503,9 +503,7 @@
       <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>﻿```
-La investigación aborda la falta de herramientas y metodologías eficaces para simular entornos de Internet de las Cosas (IoT), lo que plantea un desafío significativo para la implementación eficiente de dichos sistemas. Se propone la metodología SimulateIoT y un lenguaje específico de dominio para facilitar el diseño, generación de código y ejecución de simulaciones de entornos IoT. La metodología permite definir un entorno de simulación a través de un lenguaje especializado que utiliza técnicas de desarrollo basado en modelos, facilitando la abstracción de conceptos y proporcionando un editor gráfico para la creación de modelos. SimulateIoT se aplicó a dos estudios de caso: uno en edificios inteligentes y otro en un contexto agrícola, logrando la generación automática de código para simular sistemas y dispositivos, priorizando la conectividad y el procesamiento de datos en tiempo real. La implementación de la metodología fue validada mediante simulaciones que facilitaron la identificación de requisitos de red y almacenamiento. Este enfoque de desarrollo guiado por modelos resulta efectivo para manejar la complejidad de las tecnologías heterogéneas en el ámbito del IoT, estableciendo una base sólida para futuras mejoras y extensiones de la metodología.
-```</t>
+          <t>﻿The implementation of IoT systems encounters significant challenges due to the lack of effective tools and methodologies for simulating diverse environments. This study addresses these issues by proposing the SimulateIoT methodology, which offers a structured framework for defining and executing IoT simulation environments. By employing a Model-Driven Development (MDD) approach, the methodology facilitates the creation of a metamodel that guides the simulation process and incorporates a domain-specific language for accurate modeling. The effectiveness of SimulateIoT is demonstrated through two case studies: one focusing on smart buildings and the other on agricultural environments. Within the smart building context, the methodology improved resource efficiency through effective data management and automation; however, specific quantitative outcomes were not provided in the report. This work contributes valuable insights and tools that empower users to propose and compare various strategies prior to implementing real IoT systems, thereby enhancing their ability to analyze and understand complex IoT architectures. Ensuring stable connectivity during the simulation is crucial, although the study did not specify particular formatting constraints for the resulting reports or data presentations.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SGG: Actualizar ejemplos generados y anadir SimulateIoT como caso de prueba
Regenerados los abstracts/introducciones de Attention, Parkinson y
SimulateIoT con el pipeline actual (citas, escapado LaTeX, fusion
automatica, limite de palabras). Anadido SimulateIoT como corpus de
prueba completo: PDF principal, tres PDFs de citas (Alwasel, Calheiros,
Zeng) e introduccion original extraida para comparacion.
</commit_message>
<xml_diff>
--- a/abstracts/comparacion_abstracts.xlsx
+++ b/abstracts/comparacion_abstracts.xlsx
@@ -471,7 +471,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>﻿El artículo "Attention Is All You Need" aborda las limitaciones de las redes neuronales recurrentes (RNN) en el modelado secuencial, especialmente en tareas de traducción automática que requieren computación secuencial, lo que dificulta el paralelismo, en particular con secuencias largas. El objetivo principal de este trabajo es presentar un nuevo modelo de arquitectura denominado Transformer, que elimina la recurrencia y se basa completamente en un mecanismo de atención, mejorando así la eficiencia y la calidad en las tareas de traducción automática. La metodología adoptada incluye un modelo Transformer compuesto por secciones de codificación y decodificación apiladas, cada una de las cuales cuenta con capacidades de auto-atención y redes neuronales totalmente conectadas. Se implementó un mecanismo de atención ponderada y codificaciones posicionales para proporcionar información sobre el orden de aparición de las palabras. Los resultados muestran que el modelo Transformer alcanza un puntaje BLEU de 28.4 en la traducción inglés-alemán y 41.0 en inglés-francés, estableciendo un nuevo estado del arte. Estos logros se obtuvieron en 12 horas de entrenamiento utilizando 8 GPU P100 para el modelo básico y en 3.5 días para el modelo grande. En conclusión, el modelo Transformer no solo supera el rendimiento de modelos previos basados en RNN y estructuras convolucionales en tareas de traducción, sino que también permite un entrenamiento considerablemente más rápido al eliminar la naturaleza secuencial de los cálculos.</t>
+          <t>﻿Este trabajo aborda las limitaciones de modelos recurrentes, como RNN, LSTM y GRU, que presentan dependencias secuenciales que restringen la paralelización y reducen la eficiencia computacional, dificultando modelar dependencias a largo plazo en tareas como traducción automática. Se propone el Transformer, arquitectura que elimina la recurrencia y usa solo mecanismos de atención para capturar dependencias globales entre entradas y salidas. El Transformer usa una estructura encoder-decoder con seis capas idénticas en el modelo base, combinando atención multi-cabeza y redes feed-forward aplicadas por posición, junto con codificaciones posicionales sinusoidales que incorporan el orden sin recurrencia ni convoluciones. Se entrena con Adam y técnicas de regularización como dropout y label smoothing, usando datos masivos como el WMT 2014 para traducción inglés-alemán e inglés-francés, en hardware de 8 GPUs NVIDIA P100 durante 12 horas a 3.5 días según el tamaño. Los resultados muestran que el Transformer grande alcanza un BLEU de 28.4 en inglés-alemán, superando en más de 2 puntos a los mejores modelos previos y ensambles, y un BLEU de 41.0 en inglés-francés, mejorando modelos individuales anteriores con menor costo de entrenamiento. El modelo base también supera a competidores anteriores a menor costo. En parsing sintáctico en inglés, alcanza un F1 de hasta 92.7 en configuración semi-supervisada, superando métodos recurrentes clásicos. Experimentos con variaciones evidencian el impacto del número de cabezas y dimensiones internas en el rendimiento. En conclusión, el Transformer es el primer modelo de transducción que prescinde totalmente de recurrencia, permitiendo un entrenamiento más rápido y resultados superiores en traducción y análisis sintáctico, con perspectivas de extensión a otras modalidades y mecanismos de atención local para secuencias mayores.</t>
         </is>
       </c>
     </row>
@@ -493,7 +493,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>La Enfermedad de Parkinson (EP) es una afección crónica y progresiva que interfiere con el movimiento de los pacientes, provocando fluctuaciones en los síntomas motores y complicando su manejo y seguimiento. La evaluación actual de estos síntomas se basa en autoevaluaciones subjetivas, lo que resalta la necesidad de contar con información objetiva para mejorar el control clínico. Este estudio presenta un método innovador para identificar y clasificar las Actividades de la Vida Diaria (AVDs) en pacientes con Parkinson, utilizando Redes Neuronales Artificiales (RNA) programadas en Python. Se aplicó un Análisis de Componentes Principales (PCA) para reducir la dimensionalidad de una base de datos de 179,755 observaciones y 64 variables, recopiladas a través de sensores inerciales. Posteriormente, se entrenó un Perceptrón Multicapa (MLP) con los datos procesados, normalizando las características y utilizando la función de activación ReLU. Los resultados del modelo alcanzaron un 93% de clasificación en la medida F1-score, evidenciando una alta precisión en la identificación de AVDs, a pesar de trabajar con un conjunto de datos desbalanceado. Estos hallazgos subrayan la eficacia de las RNA combinadas con PCA y sugieren que, mediante bases de datos reducidas, es posible lograr altos niveles de precisión, proporcionando una herramienta objetiva que podría transformar la evaluación clínica en pacientes con EP.</t>
+          <t>﻿La Enfermedad de Parkinson (EP) presenta un desafío en el monitoreo efectivo debido a la dependencia de evaluaciones subjetivas. Este estudio propone un método basado en Redes Neuronales Artificiales, específicamente un Multilayer Perceptron (MLP), para clasificar seis actividades diarias relevantes en pacientes con EP utilizando señales obtenidas de sensores inerciales. Se procesaron 179,755 observaciones de tres sujetos, aplicando un filtro Butterworth y extrayendo métricas estadísticas mediante ventana móvil. Posteriormente, se empleó Análisis de Componentes Principales (PCA) para reducir la dimensionalidad conservando el 95% de la varianza, resultando en 22 componentes. El MLP, con dos capas ocultas de 16 y 10 neuronas y funciones de activación ReLU y Sigmoid, fue entrenado con el optimizador Adam durante 1000 épocas. El modelo alcanzó un F1-score del 93% en la clasificación al utilizar el conjunto completo de datos, evidenciando alta precisión. No obstante, la precisión disminuyó al 51% al entrenar con datos del 80% de los sujetos y probar con el 20% restante, mostrando limitaciones en la generalización entre individuos. La reducción dimensional facilitó la implementación en dispositivos con recursos computacionales limitados. Estos resultados respaldan la viabilidad del enfoque MLP-PCA para desarrollar sistemas objetivos de monitoreo y rehabilitación en EP, con potencial para mejorar el seguimiento clínico y la calidad de vida de los pacientes.</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,10 @@
       <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>﻿The implementation of IoT systems encounters significant challenges due to the lack of effective tools and methodologies for simulating diverse environments. This study addresses these issues by proposing the SimulateIoT methodology, which offers a structured framework for defining and executing IoT simulation environments. By employing a Model-Driven Development (MDD) approach, the methodology facilitates the creation of a metamodel that guides the simulation process and incorporates a domain-specific language for accurate modeling. The effectiveness of SimulateIoT is demonstrated through two case studies: one focusing on smart buildings and the other on agricultural environments. Within the smart building context, the methodology improved resource efficiency through effective data management and automation; however, specific quantitative outcomes were not provided in the report. This work contributes valuable insights and tools that empower users to propose and compare various strategies prior to implementing real IoT systems, thereby enhancing their ability to analyze and understand complex IoT architectures. Ensuring stable connectivity during the simulation is crucial, although the study did not specify particular formatting constraints for the resulting reports or data presentations.</t>
+          <t>﻿El presente trabajo aborda la complejidad y heterogeneidad inherente al desarrollo y simulación de entornos IoT (Internet de las Cosas), caracterizados por la diversidad de dispositivos, protocolos de comunicación y elementos de procesamiento distribuidos. Ante la falta de herramientas y metodologías que soporten el diseño, simulación y despliegue de entornos IoT completos y heterogéneos a un alto nivel de abstracción, se propone SimulateIoT, una metodología basada en técnicas de desarrollo dirigido por modelos (Model-Driven Development - MDD). Esta metodología incluye un lenguaje específico del dominio, un metamodelo, un editor gráfico y transformaciones modelo-a-texto que generan código para la simulación y el despliegue mediante microservicios encapsulados en contenedores Docker.
+El enfoque de SimulateIoT se fundamenta en una arquitectura de metamodelado de cuatro capas, definiendo conceptos de nodos (EdgeNode, FogNode, CloudNode), dispositivos, comunicación publish-subscribe, generación y procesamiento de datos (CEP/SP), almacenamiento y notificaciones. Mediante un editor gráfico basado en Eclipse GMF, los usuarios pueden definir modelos validados con reglas OCL. Posteriormente, transformaciones con Acceleo generan código que despliega nodos simulados sobre Docker Swarm, integrando brokers MQTT, bases de datos NoSQL y motores de procesamiento orientado a eventos (Esper, WSO2). La ejecución se monitoriza en tiempo real con MongoDB Compass.
+SimulateIoT se ha aplicado con éxito en dos casos de estudio: un sistema IoT para un edificio inteligente y un entorno agrícola, demostrando la modelización detallada de entornos heterogéneos, la generación y despliegue efectivos de simuladores, la capacidad de modificar modelos y regenerar código, así como la ejecución y monitorización en tiempo real. Además, se definen y ejecutan reglas complejas para el procesamiento de eventos y notificaciones. Aunque no se reportan métricas cuantitativas específicas, se valida la gestión de redes mesh y la simplificación del modelado mediante granularidades para la capacidad nodal. Se reconocen limitaciones actuales relacionadas con la movilidad nodal, simulación de hardware y conectividad, que serán abordadas en futuras extensiones.
+En conclusión, SimulateIoT demuestra que la aplicación de técnicas Model-Driven Development es una estrategia eficaz para afrontar la complejidad del diseño, simulación y despliegue de entornos IoT heterogéneos, incrementando la productividad, reduciendo errores y facilitando la validación previa a la implementación real, con soporte para arquitecturas escalables basadas en microservicios y contenedores.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SGG: Anadir cabecera a los originales de SimulateIoT y regenerar Excel de comparacion
Los ficheros de SimulateIoT no tenian titulo ni seccion "## Abstract/Introduccion
original", por lo que comparacion.py dejaba esas filas vacias en el Excel.
</commit_message>
<xml_diff>
--- a/abstracts/comparacion_abstracts.xlsx
+++ b/abstracts/comparacion_abstracts.xlsx
@@ -498,9 +498,21 @@
       </c>
     </row>
     <row r="4" ht="200" customHeight="1">
-      <c r="A4" s="2" t="inlineStr"/>
-      <c r="B4" s="2" t="inlineStr"/>
-      <c r="C4" s="2" t="inlineStr"/>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>SimulateIoT: Domain Specific Language to Design, Code Generation and Execute IoT Simulation Environments</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Internet of Things (IoT) is being applied to areas as smart-cities, home environment, agriculture, industry, etc. Developing, deploying and testing IoT projects require high investments on devices, fog nodes, cloud nodes, analytic nodes, hardware and software. New projects require high investments on devices, fog nodes, cloud nodes, analytic nodes, hardware and software before each system can be developed. In addition, the systems should be developed to test them, which implies time, effort and development costs. However, in order to decrease the cost associated to develop and test the system the IoT system can be simulated. Thus, simulating environments help to model the system, reasoning about it, and take advantage of the knowledge obtained to optimize it. Designing IoT simulation environments has been tackled focusing on low level aspects such as networks, motes and so on more than focusing on the high level concepts related to IoT environments. Additionally, the simulation users require high IoT knowledge and usually programming capabilities in order to implement the IoT environment simulation. The concepts to manage in an IoT simulation includes the common layers of an IoT environment including Edge, Fog and Cloud computing and heterogeneous technology. Model-driven development is an emerging software engineering area which aims to develop the software systems from domain models which capture at high level the domain concepts and relationships, generating from them the software artefacts by using code-generators. In this paper, a model-driven development approach has been developed to define, generate code and deploy IoT systems simulation. This approach makes it possible to design complex IoT simulation environments and deploy them without writing code. To do this, a domain metamodel, a graphical concrete syntax and a model to text transformation have been developed. The IoT simulation environment generated from each model includes the sensors, actuators, fog nodes, cloud nodes and analytical characteristics, which are deployed as microservices and Docker containers and where elements are connected by using publish-subscribe communication protocol. Additionally, two case studies, focused on smart building and agriculture IoT environments, are presented to show the simulation expressiveness.</t>
+        </is>
+      </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
           <t>﻿El presente trabajo aborda la complejidad y heterogeneidad inherente al desarrollo y simulación de entornos IoT (Internet de las Cosas), caracterizados por la diversidad de dispositivos, protocolos de comunicación y elementos de procesamiento distribuidos. Ante la falta de herramientas y metodologías que soporten el diseño, simulación y despliegue de entornos IoT completos y heterogéneos a un alto nivel de abstracción, se propone SimulateIoT, una metodología basada en técnicas de desarrollo dirigido por modelos (Model-Driven Development - MDD). Esta metodología incluye un lenguaje específico del dominio, un metamodelo, un editor gráfico y transformaciones modelo-a-texto que generan código para la simulación y el despliegue mediante microservicios encapsulados en contenedores Docker.

</xml_diff>

<commit_message>
SGG: Renombrar el proyecto de Abstrack a PaperCrew
</commit_message>
<xml_diff>
--- a/abstracts/comparacion_abstracts.xlsx
+++ b/abstracts/comparacion_abstracts.xlsx
@@ -471,7 +471,9 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>﻿Este trabajo aborda las limitaciones de modelos recurrentes, como RNN, LSTM y GRU, que presentan dependencias secuenciales que restringen la paralelización y reducen la eficiencia computacional, dificultando modelar dependencias a largo plazo en tareas como traducción automática. Se propone el Transformer, arquitectura que elimina la recurrencia y usa solo mecanismos de atención para capturar dependencias globales entre entradas y salidas. El Transformer usa una estructura encoder-decoder con seis capas idénticas en el modelo base, combinando atención multi-cabeza y redes feed-forward aplicadas por posición, junto con codificaciones posicionales sinusoidales que incorporan el orden sin recurrencia ni convoluciones. Se entrena con Adam y técnicas de regularización como dropout y label smoothing, usando datos masivos como el WMT 2014 para traducción inglés-alemán e inglés-francés, en hardware de 8 GPUs NVIDIA P100 durante 12 horas a 3.5 días según el tamaño. Los resultados muestran que el Transformer grande alcanza un BLEU de 28.4 en inglés-alemán, superando en más de 2 puntos a los mejores modelos previos y ensambles, y un BLEU de 41.0 en inglés-francés, mejorando modelos individuales anteriores con menor costo de entrenamiento. El modelo base también supera a competidores anteriores a menor costo. En parsing sintáctico en inglés, alcanza un F1 de hasta 92.7 en configuración semi-supervisada, superando métodos recurrentes clásicos. Experimentos con variaciones evidencian el impacto del número de cabezas y dimensiones internas en el rendimiento. En conclusión, el Transformer es el primer modelo de transducción que prescinde totalmente de recurrencia, permitiendo un entrenamiento más rápido y resultados superiores en traducción y análisis sintáctico, con perspectivas de extensión a otras modalidades y mecanismos de atención local para secuencias mayores.</t>
+          <t>﻿El presente trabajo introduce el Transformer, un modelo innovador de transducción de secuencias basado exclusivamente en mecanismos de atención automática (self-attention), eliminando la dependencia de estructuras recurrentes y convolucionales comunes en tareas como la traducción automática. Esta arquitectura encoder-decoder, compuesta por capas apiladas con multi-head attention y redes feed-forward posicionales, incorpora codificación posicional mediante funciones seno y coseno para preservar el orden sin recurrencias ni convoluciones. Entrenado con los conjuntos de datos WMT 2014 en inglés-alemán e inglés-francés, y optimizado mediante Adam con estrategias de tasa de aprendizaje y regularización como dropout y label smoothing, el Transformer logra mejoras significativas en eficiencia computacional y paralelización.
+En desempeño, el modelo grande alcanzó un BLEU de 28.4 en traducción inglés-alemán, superando modelos previos, incluso ensembles, tras 3.5 días de entrenamiento usando ocho GPUs NVIDIA P100. Para inglés-francés, obtuvo un BLEU de 41.8 con menor coste. La versión base también superó modelos y ensambles existentes a menor coste. Además, el Transformer mostró capacidad de generalización en análisis sintáctico inglés, logrando resultados competitivos con pocos datos.
+Este trabajo representa la primera aproximación que usa exclusivamente atención para transducción de secuencias, permitiendo un entrenamiento más rápido y paralelo, con resultados superiores al estado del arte. Los autores plantean extender el modelo a diversas modalidades y explorar atenciones restringidas para manejar secuencias largas, así como generación menos secuencial, con código fuente disponible para facilitar la investigación continua.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SGG: Arreglo de caché de CrewAI, ya que, al hacer una llamada seguida de otra, podria sobreescribirse información no deseada.
</commit_message>
<xml_diff>
--- a/abstracts/comparacion_abstracts.xlsx
+++ b/abstracts/comparacion_abstracts.xlsx
@@ -471,9 +471,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>﻿El presente trabajo introduce el Transformer, un modelo innovador de transducción de secuencias basado exclusivamente en mecanismos de atención automática (self-attention), eliminando la dependencia de estructuras recurrentes y convolucionales comunes en tareas como la traducción automática. Esta arquitectura encoder-decoder, compuesta por capas apiladas con multi-head attention y redes feed-forward posicionales, incorpora codificación posicional mediante funciones seno y coseno para preservar el orden sin recurrencias ni convoluciones. Entrenado con los conjuntos de datos WMT 2014 en inglés-alemán e inglés-francés, y optimizado mediante Adam con estrategias de tasa de aprendizaje y regularización como dropout y label smoothing, el Transformer logra mejoras significativas en eficiencia computacional y paralelización.
-En desempeño, el modelo grande alcanzó un BLEU de 28.4 en traducción inglés-alemán, superando modelos previos, incluso ensembles, tras 3.5 días de entrenamiento usando ocho GPUs NVIDIA P100. Para inglés-francés, obtuvo un BLEU de 41.8 con menor coste. La versión base también superó modelos y ensambles existentes a menor coste. Además, el Transformer mostró capacidad de generalización en análisis sintáctico inglés, logrando resultados competitivos con pocos datos.
-Este trabajo representa la primera aproximación que usa exclusivamente atención para transducción de secuencias, permitiendo un entrenamiento más rápido y paralelo, con resultados superiores al estado del arte. Los autores plantean extender el modelo a diversas modalidades y explorar atenciones restringidas para manejar secuencias largas, así como generación menos secuencial, con código fuente disponible para facilitar la investigación continua.</t>
+          <t>﻿The Transformer model addresses the limitations of traditional recurrent and convolutional neural networks in sequence modeling, particularly their sequential nature that hinders parallelization and the modeling of long-range dependencies. To overcome these challenges, the Transformer replaces recurrence entirely with a self-attention mechanism, enabling significant parallelization during training and achieving state-of-the-art results in sequence transduction tasks such as machine translation. It employs an encoder-decoder architecture with six identical layers in the base version, each containing multi-head attention mechanisms and position-wise feed-forward networks. Positional information is incorporated via sinusoidal positional encodings, compensating for the absence of recurrence and convolution. Training was conducted on the WMT 2014 English-German and English-French datasets, using byte-pair encoding and word-piece vocabularies, optimized with the Adam algorithm and regularized through label smoothing and dropout. Experiments assessed variations in attention heads, key and value dimensions, and dropout rates, and included application to English syntactic parsing. The large Transformer achieved BLEU scores of 28.4 on English-German and 41.0 on English-French translation tasks, surpassing prior state-of-the-art models by over 2 BLEU points and with markedly lower computational costs. The base model also outperformed other models and ensembles at lower training expense. Additionally, the Transformer attained strong results in English constituency parsing with F1 scores up to 92.7. This architecture enables faster training through parallelization, effectively captures long-range dependencies with reduced computational cost, and shows promise for extension to modalities beyond text, including images, audio, and video, as well as for non-sequential generation tasks.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SGG: Igualar todos los casos de prueba al idioma del paper original
- SimulateIoT y BERT regenerados en ingles (antes salian en espanol,
  no coincidian con el idioma del paper real).
- Anadidos los textos reales de abstract e introduccion de BERT
  (extraidos del PDF) para poder comparar real vs generado.
- Preparado papers/sin_abstract/bert.pdf (abstract redactado) y
  papers/sin_introduccion/redes_neuronales_parkinson.pdf (introduccion
  redactada) para completar los casos que faltaban.
- Generada la introduccion de Parkinson (antes solo existia el
  abstract) junto con su texto real de referencia.

Los 4 casos de prueba (Attention, BERT, Parkinson, SimulateIoT) quedan
ahora completos en abstract + introduccion, real + generado, en el
idioma del paper original.
</commit_message>
<xml_diff>
--- a/abstracts/comparacion_abstracts.xlsx
+++ b/abstracts/comparacion_abstracts.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -478,47 +478,67 @@
     <row r="3" ht="200" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Aplicación de Redes Neuronales Artificiales para la Clasificación de Actividades de la Vida Diaria en Sujetos con Enfermedad de Párkinson</t>
+          <t>BERT: Pre-training of Deep Bidirectional Transformers for Language Understanding</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Español</t>
+          <t>Inglés</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>El presente trabajo es un seguimiento a la propuesta para la contribución con especialistas en la salud para enriquecer los sistemas de seguimiento y apoyo en pacientes con Enfermedad de Párkinson a través de la clasificación de actividades de la vida diaria (AVDs) utilizando Redes Neuronales Artificiales programadas en lenguaje Python. El método propuesto de aprendizaje supervisado permitió la clasificación de 6 AVDs mediante 22 señales procedentes de haber aplicado Análisis de Componentes Principales; conformando la base de datos utilizada para entrenar un Perceptrón Multicapa, logrando un acercamiento a la clasificación con el 93% de medida F1-score. El presente estudio demuestra la versatilidad de las RNA basadas en MLP combinadas con la técnica de PCA, pues incluso en una base de datos desbalanceada como la utilizada permite alcanzar excelentes valores en la medida F1-score. El uso de Inteligencia Artificial y otras herramientas aplicadas en este trabajo pueden eventualmente ayudar a especialistas a desempeñar una evaluación más certera en el monitoreo de la rehabilitación en pacientes con enfermedad de Párkinson mejorando los registros y así evitar subjetividad en la interpretación de los resultados del tratamiento.</t>
+          <t>We introduce a new language representation model called BERT, which stands for Bidirectional Encoder Representations from Transformers. Unlike recent language representation models (Peters et al., 2018a; Radford et al., 2018), BERT is designed to pre-train deep bidirectional representations from unlabeled text by jointly conditioning on both left and right context in all layers. As a result, the pre-trained BERT model can be fine-tuned with just one additional output layer to create state-of-the-art models for a wide range of tasks, such as question answering and language inference, without substantial task-specific architecture modifications.
+BERT is conceptually simple and empirically powerful. It obtains new state-of-the-art results on eleven natural language processing tasks, including pushing the GLUE score to 80.5% (7.7% point absolute improvement), MultiNLI accuracy to 86.7% (4.6% absolute improvement), SQuAD v1.1 question answering Test F1 to 93.2 (1.5 point absolute improvement) and SQuAD v2.0 Test F1 to 83.1 (5.1 point absolute improvement).</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>﻿La Enfermedad de Parkinson (EP) presenta un desafío en el monitoreo efectivo debido a la dependencia de evaluaciones subjetivas. Este estudio propone un método basado en Redes Neuronales Artificiales, específicamente un Multilayer Perceptron (MLP), para clasificar seis actividades diarias relevantes en pacientes con EP utilizando señales obtenidas de sensores inerciales. Se procesaron 179,755 observaciones de tres sujetos, aplicando un filtro Butterworth y extrayendo métricas estadísticas mediante ventana móvil. Posteriormente, se empleó Análisis de Componentes Principales (PCA) para reducir la dimensionalidad conservando el 95% de la varianza, resultando en 22 componentes. El MLP, con dos capas ocultas de 16 y 10 neuronas y funciones de activación ReLU y Sigmoid, fue entrenado con el optimizador Adam durante 1000 épocas. El modelo alcanzó un F1-score del 93% en la clasificación al utilizar el conjunto completo de datos, evidenciando alta precisión. No obstante, la precisión disminuyó al 51% al entrenar con datos del 80% de los sujetos y probar con el 20% restante, mostrando limitaciones en la generalización entre individuos. La reducción dimensional facilitó la implementación en dispositivos con recursos computacionales limitados. Estos resultados respaldan la viabilidad del enfoque MLP-PCA para desarrollar sistemas objetivos de monitoreo y rehabilitación en EP, con potencial para mejorar el seguimiento clínico y la calidad de vida de los pacientes.</t>
+          <t>﻿This paper addresses the challenge of improving natural language representation learning by pretraining deep, bidirectional language models that overcome the limitations of unidirectional or shallow concatenation-based approaches. We propose and evaluate BERT (Bidirectional Encoder Representations from Transformers), a model based on a bidirectional Transformer pretrained on two unsupervised tasks: masked language modeling (MLM), where 15% of input tokens are randomly masked and predicted from both directions, and next sentence prediction (NSP), which models relationships between sentence pairs. Pretraining used large corpora, including BooksCorpus and English Wikipedia, with two model sizes: BERT BASE (12 layers, 768 hidden units, 110 million parameters) and BERT LARGE (24 layers, 1024 hidden units, 340 million parameters). We fine-tuned all model parameters on diverse NLP benchmarks such as GLUE, SQuAD v1.1 and v2.0, and SWAG, and compared with a feature-based approach using fixed BERT embeddings. Results demonstrate significant improvements over previous state-of-the-art models, with BERT LARGE achieving up to a 7-point average accuracy increase, 82.1% on GLUE, and an F1 score of 91.0% on SQuAD v1.1—surpassing prior best systems by notable margins. NSP accuracy reached 97–98%. Ablation studies confirm the importance of both pretraining tasks and model size. The feature-based approach also achieves competitive results with minimal fine-tuning. This work establishes that deep bidirectional pretraining with MLM and NSP produces richer, more generalizable language representations, enhancing performance across a broad range of NLP tasks while simplifying task-specific architectures.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="200" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>Aplicación de Redes Neuronales Artificiales para la Clasificación de Actividades de la Vida Diaria en Sujetos con Enfermedad de Párkinson</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Español</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>El presente trabajo es un seguimiento a la propuesta para la contribución con especialistas en la salud para enriquecer los sistemas de seguimiento y apoyo en pacientes con Enfermedad de Párkinson a través de la clasificación de actividades de la vida diaria (AVDs) utilizando Redes Neuronales Artificiales programadas en lenguaje Python. El método propuesto de aprendizaje supervisado permitió la clasificación de 6 AVDs mediante 22 señales procedentes de haber aplicado Análisis de Componentes Principales; conformando la base de datos utilizada para entrenar un Perceptrón Multicapa, logrando un acercamiento a la clasificación con el 93% de medida F1-score. El presente estudio demuestra la versatilidad de las RNA basadas en MLP combinadas con la técnica de PCA, pues incluso en una base de datos desbalanceada como la utilizada permite alcanzar excelentes valores en la medida F1-score. El uso de Inteligencia Artificial y otras herramientas aplicadas en este trabajo pueden eventualmente ayudar a especialistas a desempeñar una evaluación más certera en el monitoreo de la rehabilitación en pacientes con enfermedad de Párkinson mejorando los registros y así evitar subjetividad en la interpretación de los resultados del tratamiento.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>﻿La Enfermedad de Parkinson (EP) presenta un desafío en el monitoreo efectivo debido a la dependencia de evaluaciones subjetivas. Este estudio propone un método basado en Redes Neuronales Artificiales, específicamente un Multilayer Perceptron (MLP), para clasificar seis actividades diarias relevantes en pacientes con EP utilizando señales obtenidas de sensores inerciales. Se procesaron 179,755 observaciones de tres sujetos, aplicando un filtro Butterworth y extrayendo métricas estadísticas mediante ventana móvil. Posteriormente, se empleó Análisis de Componentes Principales (PCA) para reducir la dimensionalidad conservando el 95% de la varianza, resultando en 22 componentes. El MLP, con dos capas ocultas de 16 y 10 neuronas y funciones de activación ReLU y Sigmoid, fue entrenado con el optimizador Adam durante 1000 épocas. El modelo alcanzó un F1-score del 93% en la clasificación al utilizar el conjunto completo de datos, evidenciando alta precisión. No obstante, la precisión disminuyó al 51% al entrenar con datos del 80% de los sujetos y probar con el 20% restante, mostrando limitaciones en la generalización entre individuos. La reducción dimensional facilitó la implementación en dispositivos con recursos computacionales limitados. Estos resultados respaldan la viabilidad del enfoque MLP-PCA para desarrollar sistemas objetivos de monitoreo y rehabilitación en EP, con potencial para mejorar el seguimiento clínico y la calidad de vida de los pacientes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="200" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
           <t>SimulateIoT: Domain Specific Language to Design, Code Generation and Execute IoT Simulation Environments</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Inglés</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Internet of Things (IoT) is being applied to areas as smart-cities, home environment, agriculture, industry, etc. Developing, deploying and testing IoT projects require high investments on devices, fog nodes, cloud nodes, analytic nodes, hardware and software. New projects require high investments on devices, fog nodes, cloud nodes, analytic nodes, hardware and software before each system can be developed. In addition, the systems should be developed to test them, which implies time, effort and development costs. However, in order to decrease the cost associated to develop and test the system the IoT system can be simulated. Thus, simulating environments help to model the system, reasoning about it, and take advantage of the knowledge obtained to optimize it. Designing IoT simulation environments has been tackled focusing on low level aspects such as networks, motes and so on more than focusing on the high level concepts related to IoT environments. Additionally, the simulation users require high IoT knowledge and usually programming capabilities in order to implement the IoT environment simulation. The concepts to manage in an IoT simulation includes the common layers of an IoT environment including Edge, Fog and Cloud computing and heterogeneous technology. Model-driven development is an emerging software engineering area which aims to develop the software systems from domain models which capture at high level the domain concepts and relationships, generating from them the software artefacts by using code-generators. In this paper, a model-driven development approach has been developed to define, generate code and deploy IoT systems simulation. This approach makes it possible to design complex IoT simulation environments and deploy them without writing code. To do this, a domain metamodel, a graphical concrete syntax and a model to text transformation have been developed. The IoT simulation environment generated from each model includes the sensors, actuators, fog nodes, cloud nodes and analytical characteristics, which are deployed as microservices and Docker containers and where elements are connected by using publish-subscribe communication protocol. Additionally, two case studies, focused on smart building and agriculture IoT environments, are presented to show the simulation expressiveness.</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>﻿El presente trabajo aborda la complejidad y heterogeneidad inherente al desarrollo y simulación de entornos IoT (Internet de las Cosas), caracterizados por la diversidad de dispositivos, protocolos de comunicación y elementos de procesamiento distribuidos. Ante la falta de herramientas y metodologías que soporten el diseño, simulación y despliegue de entornos IoT completos y heterogéneos a un alto nivel de abstracción, se propone SimulateIoT, una metodología basada en técnicas de desarrollo dirigido por modelos (Model-Driven Development - MDD). Esta metodología incluye un lenguaje específico del dominio, un metamodelo, un editor gráfico y transformaciones modelo-a-texto que generan código para la simulación y el despliegue mediante microservicios encapsulados en contenedores Docker.
-El enfoque de SimulateIoT se fundamenta en una arquitectura de metamodelado de cuatro capas, definiendo conceptos de nodos (EdgeNode, FogNode, CloudNode), dispositivos, comunicación publish-subscribe, generación y procesamiento de datos (CEP/SP), almacenamiento y notificaciones. Mediante un editor gráfico basado en Eclipse GMF, los usuarios pueden definir modelos validados con reglas OCL. Posteriormente, transformaciones con Acceleo generan código que despliega nodos simulados sobre Docker Swarm, integrando brokers MQTT, bases de datos NoSQL y motores de procesamiento orientado a eventos (Esper, WSO2). La ejecución se monitoriza en tiempo real con MongoDB Compass.
-SimulateIoT se ha aplicado con éxito en dos casos de estudio: un sistema IoT para un edificio inteligente y un entorno agrícola, demostrando la modelización detallada de entornos heterogéneos, la generación y despliegue efectivos de simuladores, la capacidad de modificar modelos y regenerar código, así como la ejecución y monitorización en tiempo real. Además, se definen y ejecutan reglas complejas para el procesamiento de eventos y notificaciones. Aunque no se reportan métricas cuantitativas específicas, se valida la gestión de redes mesh y la simplificación del modelado mediante granularidades para la capacidad nodal. Se reconocen limitaciones actuales relacionadas con la movilidad nodal, simulación de hardware y conectividad, que serán abordadas en futuras extensiones.
-En conclusión, SimulateIoT demuestra que la aplicación de técnicas Model-Driven Development es una estrategia eficaz para afrontar la complejidad del diseño, simulación y despliegue de entornos IoT heterogéneos, incrementando la productividad, reduciendo errores y facilitando la validación previa a la implementación real, con soporte para arquitecturas escalables basadas en microservicios y contenedores.</t>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>﻿The Internet of Things (IoT) spans diverse sectors but faces challenges due to technological heterogeneity and costly deployments. This work presents SimulateIoT, a Model-Driven Development (MDD) methodology and toolset for designing, generating, and executing IoT simulations using high-level domain concepts and distributed microservice deployments. The SimulateIoT metamodel formalizes key IoT elements, including Edge, Fog, and Cloud nodes, sensors, actuators, publish-subscribe topics, synthetic and file-based data sources, Complex Event Processing (CEP) engines, NoSQL storage, notifications, and real-time rules. Models created with an EMF/GMF graphical editor and validated by OCL constraints are transformed via Acceleo into Java Thorntail microservices, Mosquitto MQTT brokers, MongoDB databases, CEP engines (Esper, WSO2), and REST APIs. Simulations are orchestrated through Docker Swarm for distributed execution. Two case studies—a smart building and an agricultural environment—demonstrate the platform’s ability to simulate sensor-actuator interactions, CEP rules, data persistence, and system orchestration. The system offers detailed monitoring of CPU, memory, and network resources. SimulateIoT enables scalable, technology-agnostic IoT modeling that streamlines system design, validation, and deployment compared to ad-hoc approaches. Limitations include partial node mobility support, a fixed domain-specific language, simplified hardware abstractions, and static configuration models; planned enhancements aim to introduce dynamic adaptive behaviors. This framework provides a robust foundation for both professional and educational IoT simulation needs.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizar develop con el estado completo de feature/abstrack
Trae el contenido de feature/abstrack (renombrado a PaperCrew, pipelines
de abstract e introduccion completos, casos de prueba BERT/SimulateIoT/
Parkinson, limpieza de boilerplate de CrewAI) sobre la version anterior
mergeada en develop (299dc20), que habia quedado desactualizada.
</commit_message>
<xml_diff>
--- a/abstracts/comparacion_abstracts.xlsx
+++ b/abstracts/comparacion_abstracts.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -471,56 +471,74 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>﻿El presente trabajo introduce el Transformer, un modelo innovador de transducción de secuencias basado exclusivamente en mecanismos de atención automática (self-attention), eliminando la dependencia de estructuras recurrentes y convolucionales comunes en tareas como la traducción automática. Esta arquitectura encoder-decoder, compuesta por capas apiladas con multi-head attention y redes feed-forward posicionales, incorpora codificación posicional mediante funciones seno y coseno para preservar el orden sin recurrencias ni convoluciones. Entrenado con los conjuntos de datos WMT 2014 en inglés-alemán e inglés-francés, y optimizado mediante Adam con estrategias de tasa de aprendizaje y regularización como dropout y label smoothing, el Transformer logra mejoras significativas en eficiencia computacional y paralelización.
-En desempeño, el modelo grande alcanzó un BLEU de 28.4 en traducción inglés-alemán, superando modelos previos, incluso ensembles, tras 3.5 días de entrenamiento usando ocho GPUs NVIDIA P100. Para inglés-francés, obtuvo un BLEU de 41.8 con menor coste. La versión base también superó modelos y ensambles existentes a menor coste. Además, el Transformer mostró capacidad de generalización en análisis sintáctico inglés, logrando resultados competitivos con pocos datos.
-Este trabajo representa la primera aproximación que usa exclusivamente atención para transducción de secuencias, permitiendo un entrenamiento más rápido y paralelo, con resultados superiores al estado del arte. Los autores plantean extender el modelo a diversas modalidades y explorar atenciones restringidas para manejar secuencias largas, así como generación menos secuencial, con código fuente disponible para facilitar la investigación continua.</t>
+          <t>﻿The Transformer model addresses the limitations of traditional recurrent and convolutional neural networks in sequence modeling, particularly their sequential nature that hinders parallelization and the modeling of long-range dependencies. To overcome these challenges, the Transformer replaces recurrence entirely with a self-attention mechanism, enabling significant parallelization during training and achieving state-of-the-art results in sequence transduction tasks such as machine translation. It employs an encoder-decoder architecture with six identical layers in the base version, each containing multi-head attention mechanisms and position-wise feed-forward networks. Positional information is incorporated via sinusoidal positional encodings, compensating for the absence of recurrence and convolution. Training was conducted on the WMT 2014 English-German and English-French datasets, using byte-pair encoding and word-piece vocabularies, optimized with the Adam algorithm and regularized through label smoothing and dropout. Experiments assessed variations in attention heads, key and value dimensions, and dropout rates, and included application to English syntactic parsing. The large Transformer achieved BLEU scores of 28.4 on English-German and 41.0 on English-French translation tasks, surpassing prior state-of-the-art models by over 2 BLEU points and with markedly lower computational costs. The base model also outperformed other models and ensembles at lower training expense. Additionally, the Transformer attained strong results in English constituency parsing with F1 scores up to 92.7. This architecture enables faster training through parallelization, effectively captures long-range dependencies with reduced computational cost, and shows promise for extension to modalities beyond text, including images, audio, and video, as well as for non-sequential generation tasks.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="200" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Aplicación de Redes Neuronales Artificiales para la Clasificación de Actividades de la Vida Diaria en Sujetos con Enfermedad de Párkinson</t>
+          <t>BERT: Pre-training of Deep Bidirectional Transformers for Language Understanding</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Español</t>
+          <t>Inglés</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>El presente trabajo es un seguimiento a la propuesta para la contribución con especialistas en la salud para enriquecer los sistemas de seguimiento y apoyo en pacientes con Enfermedad de Párkinson a través de la clasificación de actividades de la vida diaria (AVDs) utilizando Redes Neuronales Artificiales programadas en lenguaje Python. El método propuesto de aprendizaje supervisado permitió la clasificación de 6 AVDs mediante 22 señales procedentes de haber aplicado Análisis de Componentes Principales; conformando la base de datos utilizada para entrenar un Perceptrón Multicapa, logrando un acercamiento a la clasificación con el 93% de medida F1-score. El presente estudio demuestra la versatilidad de las RNA basadas en MLP combinadas con la técnica de PCA, pues incluso en una base de datos desbalanceada como la utilizada permite alcanzar excelentes valores en la medida F1-score. El uso de Inteligencia Artificial y otras herramientas aplicadas en este trabajo pueden eventualmente ayudar a especialistas a desempeñar una evaluación más certera en el monitoreo de la rehabilitación en pacientes con enfermedad de Párkinson mejorando los registros y así evitar subjetividad en la interpretación de los resultados del tratamiento.</t>
+          <t>We introduce a new language representation model called BERT, which stands for Bidirectional Encoder Representations from Transformers. Unlike recent language representation models (Peters et al., 2018a; Radford et al., 2018), BERT is designed to pre-train deep bidirectional representations from unlabeled text by jointly conditioning on both left and right context in all layers. As a result, the pre-trained BERT model can be fine-tuned with just one additional output layer to create state-of-the-art models for a wide range of tasks, such as question answering and language inference, without substantial task-specific architecture modifications.
+BERT is conceptually simple and empirically powerful. It obtains new state-of-the-art results on eleven natural language processing tasks, including pushing the GLUE score to 80.5% (7.7% point absolute improvement), MultiNLI accuracy to 86.7% (4.6% absolute improvement), SQuAD v1.1 question answering Test F1 to 93.2 (1.5 point absolute improvement) and SQuAD v2.0 Test F1 to 83.1 (5.1 point absolute improvement).</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>﻿La Enfermedad de Parkinson (EP) presenta un desafío en el monitoreo efectivo debido a la dependencia de evaluaciones subjetivas. Este estudio propone un método basado en Redes Neuronales Artificiales, específicamente un Multilayer Perceptron (MLP), para clasificar seis actividades diarias relevantes en pacientes con EP utilizando señales obtenidas de sensores inerciales. Se procesaron 179,755 observaciones de tres sujetos, aplicando un filtro Butterworth y extrayendo métricas estadísticas mediante ventana móvil. Posteriormente, se empleó Análisis de Componentes Principales (PCA) para reducir la dimensionalidad conservando el 95% de la varianza, resultando en 22 componentes. El MLP, con dos capas ocultas de 16 y 10 neuronas y funciones de activación ReLU y Sigmoid, fue entrenado con el optimizador Adam durante 1000 épocas. El modelo alcanzó un F1-score del 93% en la clasificación al utilizar el conjunto completo de datos, evidenciando alta precisión. No obstante, la precisión disminuyó al 51% al entrenar con datos del 80% de los sujetos y probar con el 20% restante, mostrando limitaciones en la generalización entre individuos. La reducción dimensional facilitó la implementación en dispositivos con recursos computacionales limitados. Estos resultados respaldan la viabilidad del enfoque MLP-PCA para desarrollar sistemas objetivos de monitoreo y rehabilitación en EP, con potencial para mejorar el seguimiento clínico y la calidad de vida de los pacientes.</t>
+          <t>﻿This work addresses the limitations of unidirectional language models in NLP, particularly their inadequate use of bidirectional context, which hampers performance on token-level tasks like question answering. We propose BERT, a novel pretraining approach based on a deeply bidirectional Transformer that employs two unsupervised tasks: masked language modeling (MLM), masking 15% of input tokens for prediction, and next sentence prediction (NSP), a binary classification capturing inter-sentence relationships. The model is pretrained on BooksCorpus and Wikipedia, with two configurations: BERT_BASE (12 layers, 768 hidden units, 12 attention heads, 110 million parameters) and BERT_LARGE (24 layers, 1024 hidden units, 16 attention heads, 340 million parameters). Fine-tuning adds task-specific output layers and trains for 2 to 4 epochs, with a maximum input length of 512 tokens. Evaluation on GLUE, SQuAD v1.1 and v2.0, SWAG, and CoNLL-2003 shows BERT outperforms previous state-of-the-art models, achieving up to 82.1% average accuracy on GLUE, F1 scores of 90.9 and 91.8 (ensemble) on SQuAD v1.1, a +5.1 point increase on SQuAD v2.0 F1, 92.2% accuracy on SWAG, and 92.8 F1 on CoNLL-2003. Ablations confirm the essential role of bidirectional pretraining and NSP, while larger models improve performance. Compared to unidirectional models like OpenAI GPT and feature-based methods such as ELMo, BERT establishes a new paradigm for deep contextualized representation learning integrating context from both directions simultaneously, enabling a single, versatile pretrained model adaptable through simple fine-tuning across diverse NLP tasks. Training leveraged TPU resources to meet computational demands.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="200" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>Aplicación de Redes Neuronales Artificiales para la Clasificación de Actividades de la Vida Diaria en Sujetos con Enfermedad de Párkinson</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Español</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>El presente trabajo es un seguimiento a la propuesta para la contribución con especialistas en la salud para enriquecer los sistemas de seguimiento y apoyo en pacientes con Enfermedad de Párkinson a través de la clasificación de actividades de la vida diaria (AVDs) utilizando Redes Neuronales Artificiales programadas en lenguaje Python. El método propuesto de aprendizaje supervisado permitió la clasificación de 6 AVDs mediante 22 señales procedentes de haber aplicado Análisis de Componentes Principales; conformando la base de datos utilizada para entrenar un Perceptrón Multicapa, logrando un acercamiento a la clasificación con el 93% de medida F1-score. El presente estudio demuestra la versatilidad de las RNA basadas en MLP combinadas con la técnica de PCA, pues incluso en una base de datos desbalanceada como la utilizada permite alcanzar excelentes valores en la medida F1-score. El uso de Inteligencia Artificial y otras herramientas aplicadas en este trabajo pueden eventualmente ayudar a especialistas a desempeñar una evaluación más certera en el monitoreo de la rehabilitación en pacientes con enfermedad de Párkinson mejorando los registros y así evitar subjetividad en la interpretación de los resultados del tratamiento.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>﻿La Enfermedad de Parkinson (EP) presenta un desafío en el monitoreo efectivo debido a la dependencia de evaluaciones subjetivas. Este estudio propone un método basado en Redes Neuronales Artificiales, específicamente un Multilayer Perceptron (MLP), para clasificar seis actividades diarias relevantes en pacientes con EP utilizando señales obtenidas de sensores inerciales. Se procesaron 179,755 observaciones de tres sujetos, aplicando un filtro Butterworth y extrayendo métricas estadísticas mediante ventana móvil. Posteriormente, se empleó Análisis de Componentes Principales (PCA) para reducir la dimensionalidad conservando el 95% de la varianza, resultando en 22 componentes. El MLP, con dos capas ocultas de 16 y 10 neuronas y funciones de activación ReLU y Sigmoid, fue entrenado con el optimizador Adam durante 1000 épocas. El modelo alcanzó un F1-score del 93% en la clasificación al utilizar el conjunto completo de datos, evidenciando alta precisión. No obstante, la precisión disminuyó al 51% al entrenar con datos del 80% de los sujetos y probar con el 20% restante, mostrando limitaciones en la generalización entre individuos. La reducción dimensional facilitó la implementación en dispositivos con recursos computacionales limitados. Estos resultados respaldan la viabilidad del enfoque MLP-PCA para desarrollar sistemas objetivos de monitoreo y rehabilitación en EP, con potencial para mejorar el seguimiento clínico y la calidad de vida de los pacientes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="200" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
           <t>SimulateIoT: Domain Specific Language to Design, Code Generation and Execute IoT Simulation Environments</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Inglés</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Internet of Things (IoT) is being applied to areas as smart-cities, home environment, agriculture, industry, etc. Developing, deploying and testing IoT projects require high investments on devices, fog nodes, cloud nodes, analytic nodes, hardware and software. New projects require high investments on devices, fog nodes, cloud nodes, analytic nodes, hardware and software before each system can be developed. In addition, the systems should be developed to test them, which implies time, effort and development costs. However, in order to decrease the cost associated to develop and test the system the IoT system can be simulated. Thus, simulating environments help to model the system, reasoning about it, and take advantage of the knowledge obtained to optimize it. Designing IoT simulation environments has been tackled focusing on low level aspects such as networks, motes and so on more than focusing on the high level concepts related to IoT environments. Additionally, the simulation users require high IoT knowledge and usually programming capabilities in order to implement the IoT environment simulation. The concepts to manage in an IoT simulation includes the common layers of an IoT environment including Edge, Fog and Cloud computing and heterogeneous technology. Model-driven development is an emerging software engineering area which aims to develop the software systems from domain models which capture at high level the domain concepts and relationships, generating from them the software artefacts by using code-generators. In this paper, a model-driven development approach has been developed to define, generate code and deploy IoT systems simulation. This approach makes it possible to design complex IoT simulation environments and deploy them without writing code. To do this, a domain metamodel, a graphical concrete syntax and a model to text transformation have been developed. The IoT simulation environment generated from each model includes the sensors, actuators, fog nodes, cloud nodes and analytical characteristics, which are deployed as microservices and Docker containers and where elements are connected by using publish-subscribe communication protocol. Additionally, two case studies, focused on smart building and agriculture IoT environments, are presented to show the simulation expressiveness.</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>﻿El presente trabajo aborda la complejidad y heterogeneidad inherente al desarrollo y simulación de entornos IoT (Internet de las Cosas), caracterizados por la diversidad de dispositivos, protocolos de comunicación y elementos de procesamiento distribuidos. Ante la falta de herramientas y metodologías que soporten el diseño, simulación y despliegue de entornos IoT completos y heterogéneos a un alto nivel de abstracción, se propone SimulateIoT, una metodología basada en técnicas de desarrollo dirigido por modelos (Model-Driven Development - MDD). Esta metodología incluye un lenguaje específico del dominio, un metamodelo, un editor gráfico y transformaciones modelo-a-texto que generan código para la simulación y el despliegue mediante microservicios encapsulados en contenedores Docker.
-El enfoque de SimulateIoT se fundamenta en una arquitectura de metamodelado de cuatro capas, definiendo conceptos de nodos (EdgeNode, FogNode, CloudNode), dispositivos, comunicación publish-subscribe, generación y procesamiento de datos (CEP/SP), almacenamiento y notificaciones. Mediante un editor gráfico basado en Eclipse GMF, los usuarios pueden definir modelos validados con reglas OCL. Posteriormente, transformaciones con Acceleo generan código que despliega nodos simulados sobre Docker Swarm, integrando brokers MQTT, bases de datos NoSQL y motores de procesamiento orientado a eventos (Esper, WSO2). La ejecución se monitoriza en tiempo real con MongoDB Compass.
-SimulateIoT se ha aplicado con éxito en dos casos de estudio: un sistema IoT para un edificio inteligente y un entorno agrícola, demostrando la modelización detallada de entornos heterogéneos, la generación y despliegue efectivos de simuladores, la capacidad de modificar modelos y regenerar código, así como la ejecución y monitorización en tiempo real. Además, se definen y ejecutan reglas complejas para el procesamiento de eventos y notificaciones. Aunque no se reportan métricas cuantitativas específicas, se valida la gestión de redes mesh y la simplificación del modelado mediante granularidades para la capacidad nodal. Se reconocen limitaciones actuales relacionadas con la movilidad nodal, simulación de hardware y conectividad, que serán abordadas en futuras extensiones.
-En conclusión, SimulateIoT demuestra que la aplicación de técnicas Model-Driven Development es una estrategia eficaz para afrontar la complejidad del diseño, simulación y despliegue de entornos IoT heterogéneos, incrementando la productividad, reduciendo errores y facilitando la validación previa a la implementación real, con soporte para arquitecturas escalables basadas en microservicios y contenedores.</t>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>﻿The Internet of Things (IoT) spans diverse sectors but faces challenges due to technological heterogeneity and costly deployments. This work presents SimulateIoT, a Model-Driven Development (MDD) methodology and toolset for designing, generating, and executing IoT simulations using high-level domain concepts and distributed microservice deployments. The SimulateIoT metamodel formalizes key IoT elements, including Edge, Fog, and Cloud nodes, sensors, actuators, publish-subscribe topics, synthetic and file-based data sources, Complex Event Processing (CEP) engines, NoSQL storage, notifications, and real-time rules. Models created with an EMF/GMF graphical editor and validated by OCL constraints are transformed via Acceleo into Java Thorntail microservices, Mosquitto MQTT brokers, MongoDB databases, CEP engines (Esper, WSO2), and REST APIs. Simulations are orchestrated through Docker Swarm for distributed execution. Two case studies—a smart building and an agricultural environment—demonstrate the platform’s ability to simulate sensor-actuator interactions, CEP rules, data persistence, and system orchestration. The system offers detailed monitoring of CPU, memory, and network resources. SimulateIoT enables scalable, technology-agnostic IoT modeling that streamlines system design, validation, and deployment compared to ad-hoc approaches. Limitations include partial node mobility support, a fixed domain-specific language, simplified hardware abstractions, and static configuration models; planned enhancements aim to introduce dynamic adaptive behaviors. This framework provides a robust foundation for both professional and educational IoT simulation needs.</t>
         </is>
       </c>
     </row>

</xml_diff>